<commit_message>
Update Ottavia's affiliation for BBS Nextgen and recompile
</commit_message>
<xml_diff>
--- a/data/roster_nextgen.xlsx
+++ b/data/roster_nextgen.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/widmelu1/Documents/git/bbs-basel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C708B82-1E30-C14E-8B2F-4F14348D084D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70657D8-3BAB-7F44-8EE3-BE22B7F6042F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="780" windowWidth="41120" windowHeight="24180" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -612,7 +612,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E8" s="2">
         <v>1</v>

</xml_diff>